<commit_message>
Ticket for  SMASHEDLEMON45 O(n²) issue. Weird! Should match via Bracket 1 & 2 but doesn't??? CLIP called pre-brackets might be the issue (dataset huge)
</commit_message>
<xml_diff>
--- a/test/datasets/CiMini/Brackets-Complete.xlsx
+++ b/test/datasets/CiMini/Brackets-Complete.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JefB\Documents\JBGITROOT\prism\test\JBComplete\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JefB\Documents\JBGITROOT\prism\test\datasets\CiMini\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="451">
   <si>
     <t>familyID</t>
   </si>
@@ -2250,12 +2250,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -2328,76 +2322,6 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2459,8 +2383,84 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2796,993 +2796,1049 @@
   <dimension ref="A1:AF33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" style="61" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" style="61" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" style="61" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.7109375" style="61" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.85546875" style="61" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" style="61" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.85546875" style="61" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="61" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" style="61"/>
-    <col min="10" max="10" width="8.85546875" style="61" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.28515625" style="61" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.85546875" style="61" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="81.42578125" style="61" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.85546875" style="61" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.5703125" style="61" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="4.5703125" style="61" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.5703125" style="61" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.140625" style="61"/>
-    <col min="19" max="19" width="9.5703125" style="61" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="7.42578125" style="61" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.85546875" style="61" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="9.140625" style="61"/>
-    <col min="24" max="24" width="8.42578125" style="61" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.140625" style="61"/>
-    <col min="26" max="26" width="8.28515625" style="61" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13.7109375" style="61" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="7.7109375" style="61" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="21.85546875" style="61" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="6.5703125" style="61" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="6.85546875" style="61" bestFit="1" customWidth="1"/>
-    <col min="32" max="16384" width="9.140625" style="61"/>
+    <col min="1" max="1" width="14" style="33" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" style="33" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" style="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.85546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" style="33" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="33"/>
+    <col min="10" max="10" width="8.85546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" style="33" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="81.42578125" style="33" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.85546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.5703125" style="33" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.5703125" style="33" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.5703125" style="33" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" style="33"/>
+    <col min="19" max="19" width="9.5703125" style="33" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="7.42578125" style="33" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8.85546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.140625" style="33"/>
+    <col min="24" max="24" width="8.42578125" style="33" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.140625" style="33"/>
+    <col min="26" max="26" width="8.28515625" style="33" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.7109375" style="33" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="7.7109375" style="33" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21.85546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.5703125" style="33" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="6.85546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="32" max="16384" width="9.140625" style="33"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="79" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="71" t="s">
+    <row r="1" spans="1:32" s="51" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="43" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="43" t="s">
         <v>190</v>
       </c>
-      <c r="C1" s="72" t="s">
+      <c r="C1" s="44" t="s">
         <v>191</v>
       </c>
-      <c r="D1" s="71" t="s">
+      <c r="D1" s="43" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="71" t="s">
+      <c r="E1" s="43" t="s">
         <v>193</v>
       </c>
-      <c r="F1" s="71" t="s">
+      <c r="F1" s="43" t="s">
         <v>194</v>
       </c>
-      <c r="G1" s="71" t="s">
+      <c r="G1" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="71" t="s">
+      <c r="H1" s="43" t="s">
         <v>195</v>
       </c>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71" t="s">
+      <c r="I1" s="43"/>
+      <c r="J1" s="43" t="s">
         <v>196</v>
       </c>
-      <c r="K1" s="71" t="s">
+      <c r="K1" s="43" t="s">
         <v>197</v>
       </c>
-      <c r="L1" s="71" t="s">
+      <c r="L1" s="43" t="s">
         <v>198</v>
       </c>
-      <c r="M1" s="71" t="s">
+      <c r="M1" s="43" t="s">
         <v>199</v>
       </c>
-      <c r="N1" s="71" t="s">
+      <c r="N1" s="43" t="s">
         <v>200</v>
       </c>
-      <c r="O1" s="71" t="s">
+      <c r="O1" s="43" t="s">
         <v>201</v>
       </c>
-      <c r="P1" s="71" t="s">
+      <c r="P1" s="43" t="s">
         <v>202</v>
       </c>
-      <c r="Q1" s="71" t="s">
+      <c r="Q1" s="43" t="s">
         <v>203</v>
       </c>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71" t="s">
+      <c r="R1" s="43"/>
+      <c r="S1" s="43" t="s">
         <v>204</v>
       </c>
-      <c r="T1" s="71" t="s">
+      <c r="T1" s="43" t="s">
         <v>205</v>
       </c>
-      <c r="U1" s="71" t="s">
+      <c r="U1" s="43" t="s">
         <v>206</v>
       </c>
-      <c r="V1" s="71" t="s">
+      <c r="V1" s="43" t="s">
         <v>207</v>
       </c>
-      <c r="W1" s="71" t="s">
+      <c r="W1" s="43" t="s">
         <v>208</v>
       </c>
-      <c r="X1" s="71" t="s">
+      <c r="X1" s="43" t="s">
         <v>209</v>
       </c>
-      <c r="Y1" s="71"/>
-      <c r="Z1" s="73" t="s">
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="45" t="s">
         <v>210</v>
       </c>
-      <c r="AA1" s="74" t="s">
+      <c r="AA1" s="46" t="s">
         <v>211</v>
       </c>
-      <c r="AB1" s="75" t="s">
+      <c r="AB1" s="47" t="s">
         <v>212</v>
       </c>
-      <c r="AC1" s="76" t="s">
+      <c r="AC1" s="48" t="s">
         <v>213</v>
       </c>
-      <c r="AD1" s="76" t="s">
+      <c r="AD1" s="48" t="s">
         <v>214</v>
       </c>
-      <c r="AE1" s="77" t="s">
+      <c r="AE1" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="AF1" s="78" t="s">
+      <c r="AF1" s="50" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A2" s="61">
+      <c r="A2" s="33">
         <v>98884444</v>
       </c>
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="61" t="s">
+      <c r="C2" s="33" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A3" s="61">
+      <c r="A3" s="33">
         <v>98884445</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="33" t="s">
         <v>251</v>
       </c>
-      <c r="C3" s="61" t="s">
+      <c r="C3" s="33" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A4" s="61">
+      <c r="A4" s="33">
         <v>99147525</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="33" t="s">
         <v>290</v>
       </c>
-      <c r="C4" s="80">
+      <c r="C4" s="52">
         <v>8721309290498</v>
       </c>
-      <c r="E4" s="61" t="s">
+      <c r="E4" s="33" t="s">
         <v>293</v>
       </c>
-      <c r="G4" s="61" t="s">
+      <c r="G4" s="33" t="s">
         <v>292</v>
       </c>
-      <c r="H4" s="61" t="s">
+      <c r="H4" s="33" t="s">
         <v>294</v>
       </c>
-      <c r="M4" s="61" t="s">
+      <c r="M4" s="33" t="s">
         <v>295</v>
       </c>
-      <c r="N4" s="61" t="s">
+      <c r="N4" s="33" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A5" s="61">
+      <c r="A5" s="33">
         <v>99147533</v>
       </c>
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="33" t="s">
         <v>296</v>
       </c>
-      <c r="C5" s="80">
+      <c r="C5" s="52">
         <v>8721309209575</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="33" t="s">
         <v>297</v>
       </c>
-      <c r="G5" s="61" t="s">
+      <c r="G5" s="33" t="s">
         <v>292</v>
       </c>
-      <c r="H5" s="61" t="s">
+      <c r="H5" s="33" t="s">
         <v>298</v>
       </c>
-      <c r="M5" s="61" t="s">
+      <c r="M5" s="33" t="s">
         <v>295</v>
       </c>
-      <c r="N5" s="61" t="s">
+      <c r="N5" s="33" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A6" s="61">
+      <c r="A6" s="33">
         <v>90861025</v>
       </c>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="33" t="s">
         <v>301</v>
       </c>
-      <c r="C6" s="81" t="s">
+      <c r="C6" s="53" t="s">
         <v>303</v>
       </c>
-      <c r="D6" s="61" t="s">
+      <c r="D6" s="33" t="s">
         <v>304</v>
       </c>
-      <c r="E6" s="61" t="s">
+      <c r="E6" s="33" t="s">
         <v>302</v>
       </c>
-      <c r="H6" s="61" t="s">
+      <c r="H6" s="33" t="s">
         <v>308</v>
       </c>
-      <c r="K6" s="61" t="s">
+      <c r="K6" s="33" t="s">
         <v>309</v>
       </c>
-      <c r="L6" s="61" t="s">
+      <c r="L6" s="33" t="s">
         <v>307</v>
       </c>
-      <c r="Q6" s="61" t="s">
+      <c r="Q6" s="33" t="s">
         <v>311</v>
       </c>
-      <c r="AA6" s="61" t="s">
+      <c r="AA6" s="33" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A7" s="61">
+      <c r="A7" s="33">
         <v>90861026</v>
       </c>
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="33" t="s">
         <v>327</v>
       </c>
-      <c r="C7" s="81" t="s">
+      <c r="C7" s="53" t="s">
         <v>328</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="33" t="s">
         <v>329</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="33" t="s">
         <v>317</v>
       </c>
-      <c r="F7" s="82"/>
-      <c r="H7" s="61" t="s">
+      <c r="F7" s="54"/>
+      <c r="H7" s="33" t="s">
         <v>331</v>
       </c>
-      <c r="K7" s="61" t="s">
+      <c r="K7" s="33" t="s">
         <v>332</v>
       </c>
-      <c r="Q7" s="61" t="s">
+      <c r="Q7" s="33" t="s">
         <v>318</v>
       </c>
-      <c r="AA7" s="61" t="s">
+      <c r="AA7" s="33" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A8" s="61">
+      <c r="A8" s="33">
         <v>90861083</v>
       </c>
-      <c r="B8" s="61" t="s">
+      <c r="B8" s="33" t="s">
         <v>333</v>
       </c>
-      <c r="C8" s="81" t="s">
+      <c r="C8" s="53" t="s">
         <v>334</v>
       </c>
-      <c r="D8" s="61" t="s">
+      <c r="D8" s="33" t="s">
         <v>335</v>
       </c>
-      <c r="E8" s="61" t="s">
+      <c r="E8" s="33" t="s">
         <v>313</v>
       </c>
-      <c r="H8" s="61" t="s">
+      <c r="H8" s="33" t="s">
         <v>319</v>
       </c>
-      <c r="I8" s="61" t="s">
+      <c r="I8" s="33" t="s">
         <v>337</v>
       </c>
-      <c r="K8" s="61" t="s">
+      <c r="K8" s="33" t="s">
         <v>338</v>
       </c>
-      <c r="N8" s="61" t="s">
+      <c r="N8" s="33" t="s">
         <v>320</v>
       </c>
-      <c r="Q8" s="61" t="s">
+      <c r="Q8" s="33" t="s">
         <v>316</v>
       </c>
-      <c r="AA8" s="61" t="s">
+      <c r="AA8" s="33" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A9" s="61">
+      <c r="A9" s="33">
         <v>90861052</v>
       </c>
-      <c r="B9" s="61" t="s">
+      <c r="B9" s="33" t="s">
         <v>339</v>
       </c>
-      <c r="C9" s="81" t="s">
+      <c r="C9" s="53" t="s">
         <v>340</v>
       </c>
-      <c r="D9" s="61" t="s">
+      <c r="D9" s="33" t="s">
         <v>341</v>
       </c>
-      <c r="E9" s="61" t="s">
+      <c r="E9" s="33" t="s">
         <v>313</v>
       </c>
-      <c r="H9" s="61" t="s">
+      <c r="H9" s="33" t="s">
         <v>319</v>
       </c>
-      <c r="I9" s="61" t="s">
+      <c r="I9" s="33" t="s">
         <v>343</v>
       </c>
-      <c r="K9" s="61" t="s">
+      <c r="K9" s="33" t="s">
         <v>321</v>
       </c>
-      <c r="N9" s="61" t="s">
+      <c r="N9" s="33" t="s">
         <v>322</v>
       </c>
-      <c r="Q9" s="61" t="s">
+      <c r="Q9" s="33" t="s">
         <v>316</v>
       </c>
-      <c r="AA9" s="61" t="s">
+      <c r="AA9" s="33" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A10" s="80">
+      <c r="A10" s="52">
         <v>98226972</v>
       </c>
-      <c r="B10" s="80" t="s">
+      <c r="B10" s="52" t="s">
         <v>347</v>
       </c>
-      <c r="C10" s="81" t="s">
+      <c r="C10" s="53" t="s">
         <v>348</v>
       </c>
-      <c r="D10" s="80" t="s">
+      <c r="D10" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="E10" s="80" t="s">
+      <c r="E10" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="61" t="s">
+      <c r="H10" s="33" t="s">
         <v>351</v>
       </c>
-      <c r="K10" s="61" t="s">
+      <c r="K10" s="33" t="s">
         <v>352</v>
       </c>
-      <c r="N10" s="61" t="s">
+      <c r="N10" s="33" t="s">
         <v>349</v>
       </c>
-      <c r="AA10" s="61" t="s">
+      <c r="AA10" s="33" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A11" s="80">
+      <c r="A11" s="52">
         <v>98226808</v>
       </c>
-      <c r="B11" s="80" t="s">
+      <c r="B11" s="52" t="s">
         <v>344</v>
       </c>
-      <c r="C11" s="81" t="s">
+      <c r="C11" s="53" t="s">
         <v>345</v>
       </c>
-      <c r="D11" s="80" t="s">
+      <c r="D11" s="52" t="s">
         <v>353</v>
       </c>
-      <c r="E11" s="80" t="s">
+      <c r="E11" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="61" t="s">
+      <c r="H11" s="33" t="s">
         <v>355</v>
       </c>
-      <c r="K11" s="61" t="s">
+      <c r="K11" s="33" t="s">
         <v>248</v>
       </c>
-      <c r="N11" s="61" t="s">
+      <c r="N11" s="33" t="s">
         <v>349</v>
       </c>
-      <c r="AA11" s="61" t="s">
+      <c r="AA11" s="33" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A12" s="80">
+      <c r="A12" s="52">
         <v>91337133</v>
       </c>
-      <c r="B12" s="80" t="s">
+      <c r="B12" s="52" t="s">
         <v>356</v>
       </c>
-      <c r="C12" s="81">
+      <c r="C12" s="53">
         <v>4061237287825</v>
       </c>
-      <c r="D12" s="80" t="s">
+      <c r="D12" s="52" t="s">
         <v>357</v>
       </c>
-      <c r="E12" s="61" t="s">
+      <c r="E12" s="33" t="s">
         <v>359</v>
       </c>
-      <c r="G12" s="61" t="s">
+      <c r="G12" s="33" t="s">
         <v>358</v>
       </c>
-      <c r="H12" s="61" t="s">
+      <c r="H12" s="33" t="s">
         <v>360</v>
       </c>
-      <c r="K12" s="61" t="s">
+      <c r="K12" s="33" t="s">
         <v>361</v>
       </c>
-      <c r="L12" s="61" t="s">
+      <c r="L12" s="33" t="s">
         <v>362</v>
       </c>
-      <c r="AA12" s="61" t="s">
+      <c r="AA12" s="33" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A13" s="61">
+      <c r="A13" s="33">
         <v>94613033</v>
       </c>
-      <c r="B13" s="81">
+      <c r="B13" s="53">
         <v>889624293711</v>
       </c>
-      <c r="D13" s="61" t="s">
+      <c r="D13" s="33" t="s">
         <v>365</v>
       </c>
-      <c r="E13" s="61" t="s">
+      <c r="E13" s="33" t="s">
         <v>364</v>
       </c>
-      <c r="F13" s="82"/>
-      <c r="J13" s="61" t="s">
+      <c r="F13" s="54"/>
+      <c r="J13" s="33" t="s">
         <v>369</v>
       </c>
-      <c r="K13" s="61" t="s">
+      <c r="K13" s="33" t="s">
         <v>367</v>
       </c>
-      <c r="Q13" s="61" t="s">
+      <c r="Q13" s="33" t="s">
         <v>368</v>
       </c>
-      <c r="AA13" s="61" t="s">
+      <c r="AA13" s="33" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A14" s="61">
+      <c r="A14" s="33">
         <v>90861075</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="33" t="s">
         <v>370</v>
       </c>
-      <c r="C14" s="81" t="s">
+      <c r="C14" s="53" t="s">
         <v>371</v>
       </c>
-      <c r="D14" s="61" t="s">
+      <c r="D14" s="33" t="s">
         <v>372</v>
       </c>
-      <c r="E14" s="61" t="s">
+      <c r="E14" s="33" t="s">
         <v>323</v>
       </c>
-      <c r="F14" s="82"/>
-      <c r="H14" s="61" t="s">
+      <c r="F14" s="54"/>
+      <c r="H14" s="33" t="s">
         <v>323</v>
       </c>
-      <c r="I14" s="83" t="s">
+      <c r="I14" s="55" t="s">
         <v>326</v>
       </c>
-      <c r="K14" s="61" t="s">
+      <c r="K14" s="33" t="s">
         <v>321</v>
       </c>
-      <c r="N14" s="61" t="s">
+      <c r="N14" s="33" t="s">
         <v>373</v>
       </c>
-      <c r="Q14" s="61" t="s">
+      <c r="Q14" s="33" t="s">
         <v>316</v>
       </c>
-      <c r="AA14" s="61" t="s">
+      <c r="AA14" s="33" t="s">
         <v>324</v>
       </c>
-      <c r="AB14" s="61" t="s">
+      <c r="AB14" s="33" t="s">
         <v>378</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A15" s="61">
+      <c r="A15" s="33">
         <v>90861071</v>
       </c>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="33" t="s">
         <v>374</v>
       </c>
-      <c r="C15" s="81" t="s">
+      <c r="C15" s="53" t="s">
         <v>375</v>
       </c>
-      <c r="D15" s="61" t="s">
+      <c r="D15" s="33" t="s">
         <v>376</v>
       </c>
-      <c r="E15" s="61" t="s">
+      <c r="E15" s="33" t="s">
         <v>323</v>
       </c>
-      <c r="F15" s="82"/>
-      <c r="H15" s="61" t="s">
+      <c r="F15" s="54"/>
+      <c r="H15" s="33" t="s">
         <v>323</v>
       </c>
-      <c r="I15" s="83" t="s">
+      <c r="I15" s="55" t="s">
         <v>379</v>
       </c>
-      <c r="K15" s="61" t="s">
+      <c r="K15" s="33" t="s">
         <v>314</v>
       </c>
-      <c r="N15" s="61" t="s">
+      <c r="N15" s="33" t="s">
         <v>315</v>
       </c>
-      <c r="Q15" s="61" t="s">
+      <c r="Q15" s="33" t="s">
         <v>316</v>
       </c>
-      <c r="AA15" s="61" t="s">
+      <c r="AA15" s="33" t="s">
         <v>377</v>
       </c>
-      <c r="AB15" s="61" t="s">
+      <c r="AB15" s="33" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A16" s="61">
+      <c r="A16" s="33">
         <v>90861076</v>
       </c>
-      <c r="B16" s="61" t="s">
+      <c r="B16" s="33" t="s">
         <v>380</v>
       </c>
-      <c r="C16" s="81" t="s">
+      <c r="C16" s="53" t="s">
         <v>381</v>
       </c>
-      <c r="D16" s="61" t="s">
+      <c r="D16" s="33" t="s">
         <v>382</v>
       </c>
-      <c r="E16" s="61" t="s">
+      <c r="E16" s="33" t="s">
         <v>323</v>
       </c>
-      <c r="F16" s="82"/>
-      <c r="H16" s="61" t="s">
+      <c r="F16" s="54"/>
+      <c r="H16" s="33" t="s">
         <v>323</v>
       </c>
-      <c r="I16" s="83" t="s">
+      <c r="I16" s="55" t="s">
         <v>326</v>
       </c>
-      <c r="K16" s="61" t="s">
+      <c r="K16" s="33" t="s">
         <v>321</v>
       </c>
-      <c r="N16" s="61" t="s">
+      <c r="N16" s="33" t="s">
         <v>383</v>
       </c>
-      <c r="Q16" s="61" t="s">
+      <c r="Q16" s="33" t="s">
         <v>316</v>
       </c>
-      <c r="AA16" s="61" t="s">
+      <c r="AA16" s="33" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="17" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A17" s="61">
+      <c r="A17" s="33">
         <v>99985014</v>
       </c>
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="33" t="s">
         <v>385</v>
       </c>
-      <c r="C17" s="84" t="s">
+      <c r="C17" s="56" t="s">
         <v>387</v>
       </c>
-      <c r="D17" s="61" t="s">
+      <c r="D17" s="33" t="s">
         <v>384</v>
       </c>
-      <c r="E17" s="61" t="s">
+      <c r="E17" s="33" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A18" s="61">
+      <c r="A18" s="33">
         <v>98008135</v>
       </c>
-      <c r="B18" s="85" t="s">
+      <c r="B18" s="57" t="s">
         <v>388</v>
       </c>
-      <c r="D18" s="61" t="s">
+      <c r="D18" s="33" t="s">
         <v>390</v>
       </c>
-      <c r="E18" s="61" t="s">
+      <c r="E18" s="33" t="s">
         <v>392</v>
       </c>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A19" s="61">
+      <c r="A19" s="33">
         <v>98008136</v>
       </c>
-      <c r="B19" s="85" t="s">
+      <c r="B19" s="57" t="s">
         <v>389</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="33" t="s">
         <v>391</v>
       </c>
-      <c r="E19" s="61" t="s">
+      <c r="E19" s="33" t="s">
         <v>392</v>
       </c>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A20" s="80">
+      <c r="A20" s="52">
         <v>97019930</v>
       </c>
-      <c r="D20" s="61" t="s">
+      <c r="D20" s="33" t="s">
         <v>394</v>
       </c>
-      <c r="E20" s="61" t="s">
+      <c r="E20" s="33" t="s">
         <v>393</v>
       </c>
-      <c r="F20" s="61" t="s">
+      <c r="F20" s="33" t="s">
         <v>395</v>
       </c>
-      <c r="G20" s="61" t="s">
+      <c r="G20" s="33" t="s">
         <v>396</v>
       </c>
-      <c r="H20" s="61" t="s">
+      <c r="H20" s="33" t="s">
         <v>397</v>
       </c>
-      <c r="J20" s="61" t="s">
+      <c r="J20" s="33" t="s">
         <v>299</v>
       </c>
-      <c r="K20" s="61" t="s">
+      <c r="K20" s="33" t="s">
         <v>248</v>
       </c>
-      <c r="L20" s="61" t="s">
+      <c r="L20" s="33" t="s">
         <v>402</v>
       </c>
-      <c r="M20" s="61" t="s">
+      <c r="M20" s="33" t="s">
         <v>398</v>
       </c>
-      <c r="N20" s="61" t="s">
+      <c r="N20" s="33" t="s">
         <v>250</v>
       </c>
-      <c r="O20" s="61" t="s">
+      <c r="O20" s="33" t="s">
         <v>399</v>
       </c>
-      <c r="Q20" s="61" t="s">
+      <c r="Q20" s="33" t="s">
         <v>318</v>
       </c>
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A21" s="80">
+      <c r="A21" s="52">
         <v>98091311</v>
       </c>
-      <c r="D21" s="61" t="s">
+      <c r="D21" s="33" t="s">
         <v>400</v>
       </c>
-      <c r="E21" s="61" t="s">
+      <c r="E21" s="33" t="s">
         <v>393</v>
       </c>
-      <c r="F21" s="61" t="s">
+      <c r="F21" s="33" t="s">
         <v>395</v>
       </c>
-      <c r="G21" s="61" t="s">
+      <c r="G21" s="33" t="s">
         <v>396</v>
       </c>
-      <c r="H21" s="61" t="s">
+      <c r="H21" s="33" t="s">
         <v>397</v>
       </c>
-      <c r="J21" s="61" t="s">
+      <c r="J21" s="33" t="s">
         <v>299</v>
       </c>
-      <c r="K21" s="61" t="s">
+      <c r="K21" s="33" t="s">
         <v>248</v>
       </c>
-      <c r="L21" s="61" t="s">
+      <c r="L21" s="33" t="s">
         <v>401</v>
       </c>
-      <c r="M21" s="61" t="s">
+      <c r="M21" s="33" t="s">
         <v>398</v>
       </c>
-      <c r="N21" s="61" t="s">
+      <c r="N21" s="33" t="s">
         <v>403</v>
       </c>
-      <c r="O21" s="61" t="s">
+      <c r="O21" s="33" t="s">
         <v>399</v>
       </c>
-      <c r="Q21" s="61" t="s">
+      <c r="Q21" s="33" t="s">
         <v>318</v>
       </c>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A22" s="80">
+      <c r="A22" s="52">
         <v>91234321</v>
       </c>
-      <c r="D22" s="61" t="s">
+      <c r="D22" s="33" t="s">
         <v>404</v>
       </c>
-      <c r="E22" s="61" t="s">
+      <c r="E22" s="33" t="s">
         <v>393</v>
       </c>
-      <c r="F22" s="61" t="s">
+      <c r="F22" s="33" t="s">
         <v>395</v>
       </c>
-      <c r="G22" s="61" t="s">
+      <c r="G22" s="33" t="s">
         <v>396</v>
       </c>
-      <c r="H22" s="61" t="s">
+      <c r="H22" s="33" t="s">
         <v>397</v>
       </c>
-      <c r="J22" s="61" t="s">
+      <c r="J22" s="33" t="s">
         <v>299</v>
       </c>
-      <c r="K22" s="61" t="s">
+      <c r="K22" s="33" t="s">
         <v>248</v>
       </c>
-      <c r="L22" s="61" t="s">
+      <c r="L22" s="33" t="s">
         <v>405</v>
       </c>
-      <c r="M22" s="61" t="s">
+      <c r="M22" s="33" t="s">
         <v>398</v>
       </c>
-      <c r="N22" s="61" t="s">
+      <c r="N22" s="33" t="s">
         <v>406</v>
       </c>
-      <c r="O22" s="61" t="s">
+      <c r="O22" s="33" t="s">
         <v>399</v>
       </c>
-      <c r="Q22" s="61" t="s">
+      <c r="Q22" s="33" t="s">
         <v>318</v>
       </c>
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A23" s="61">
+      <c r="A23" s="33">
         <v>99984905</v>
       </c>
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="33" t="s">
         <v>408</v>
       </c>
-      <c r="C23" s="81">
+      <c r="C23" s="53">
         <v>8718679018555</v>
       </c>
-      <c r="D23" s="61" t="s">
+      <c r="D23" s="33" t="s">
         <v>407</v>
       </c>
-      <c r="E23" s="61" t="s">
+      <c r="E23" s="33" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A24" s="61">
+      <c r="A24" s="33">
         <v>99985047</v>
       </c>
-      <c r="B24" s="61" t="s">
+      <c r="B24" s="33" t="s">
         <v>410</v>
       </c>
-      <c r="C24" s="81">
+      <c r="C24" s="53">
         <v>8718679021272</v>
       </c>
-      <c r="D24" s="61" t="s">
+      <c r="D24" s="33" t="s">
         <v>409</v>
       </c>
-      <c r="E24" s="61" t="s">
+      <c r="E24" s="33" t="s">
         <v>15</v>
       </c>
+      <c r="K24" s="88"/>
+      <c r="L24" s="88"/>
+      <c r="M24" s="88"/>
+      <c r="N24" s="88"/>
+      <c r="O24" s="88"/>
+      <c r="P24" s="88"/>
+      <c r="Q24" s="88"/>
+      <c r="R24" s="88"/>
+      <c r="S24" s="88"/>
     </row>
     <row r="25" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A25" s="61">
+      <c r="A25" s="33">
         <v>98768768</v>
       </c>
-      <c r="B25" s="61" t="s">
+      <c r="B25" s="33" t="s">
         <v>414</v>
       </c>
-      <c r="C25" s="85" t="s">
+      <c r="C25" s="57" t="s">
         <v>415</v>
       </c>
-      <c r="D25" s="61" t="s">
+      <c r="D25" s="33" t="s">
         <v>411</v>
       </c>
-      <c r="G25" s="61" t="s">
+      <c r="G25" s="33" t="s">
         <v>412</v>
       </c>
-      <c r="H25" s="61" t="s">
+      <c r="H25" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="N25" s="61" t="s">
+      <c r="K25" s="88"/>
+      <c r="L25" s="88"/>
+      <c r="M25" s="88"/>
+      <c r="N25" s="88" t="s">
         <v>413</v>
       </c>
+      <c r="O25" s="88"/>
+      <c r="P25" s="88"/>
+      <c r="Q25" s="88"/>
+      <c r="R25" s="88"/>
+      <c r="S25" s="88"/>
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A26" s="80">
+      <c r="A26" s="52">
         <v>98226706</v>
       </c>
-      <c r="B26" s="80" t="s">
+      <c r="B26" s="52" t="s">
         <v>416</v>
       </c>
-      <c r="C26" s="81" t="s">
+      <c r="C26" s="53" t="s">
         <v>417</v>
       </c>
-      <c r="D26" s="86"/>
-      <c r="E26" s="61" t="s">
+      <c r="D26" s="58"/>
+      <c r="E26" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G26" s="61" t="s">
+      <c r="G26" s="33" t="s">
         <v>412</v>
       </c>
-      <c r="H26" s="61" t="s">
+      <c r="H26" s="33" t="s">
         <v>418</v>
       </c>
-      <c r="L26" s="87"/>
-      <c r="M26" s="87"/>
-      <c r="N26" s="87"/>
-      <c r="O26" s="87"/>
-      <c r="P26" s="87"/>
-      <c r="Q26" s="87"/>
+      <c r="K26" s="88"/>
+      <c r="L26" s="88"/>
+      <c r="M26" s="88"/>
+      <c r="N26" s="88"/>
+      <c r="O26" s="88"/>
+      <c r="P26" s="88"/>
+      <c r="Q26" s="88"/>
+      <c r="R26" s="88"/>
+      <c r="S26" s="88"/>
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A27" s="61">
+      <c r="A27" s="33">
         <v>98636325</v>
       </c>
-      <c r="B27" s="61" t="s">
+      <c r="B27" s="33" t="s">
         <v>419</v>
       </c>
-      <c r="C27" s="61">
+      <c r="C27" s="33">
         <v>8719558938070</v>
       </c>
-      <c r="D27" s="61" t="s">
+      <c r="D27" s="33" t="s">
         <v>421</v>
       </c>
-      <c r="E27" s="61" t="s">
+      <c r="E27" s="33" t="s">
         <v>420</v>
       </c>
-      <c r="H27" s="61" t="s">
+      <c r="H27" s="33" t="s">
         <v>422</v>
       </c>
-      <c r="J27" s="61" t="s">
+      <c r="J27" s="33" t="s">
         <v>424</v>
       </c>
-      <c r="K27" s="61" t="s">
+      <c r="K27" s="88" t="s">
         <v>425</v>
       </c>
-      <c r="L27" s="61" t="s">
+      <c r="L27" s="88" t="s">
         <v>423</v>
       </c>
-      <c r="N27" s="61" t="s">
+      <c r="M27" s="88"/>
+      <c r="N27" s="88" t="s">
         <v>426</v>
       </c>
-      <c r="Z27" s="88" t="s">
+      <c r="O27" s="88"/>
+      <c r="P27" s="88"/>
+      <c r="Q27" s="88"/>
+      <c r="R27" s="88"/>
+      <c r="S27" s="88"/>
+      <c r="Z27" s="59" t="s">
         <v>427</v>
       </c>
-      <c r="AF27" s="61" t="s">
+      <c r="AF27" s="33" t="s">
         <v>428</v>
       </c>
     </row>
     <row r="28" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A28" s="61">
+      <c r="A28" s="33">
         <v>98636303</v>
       </c>
-      <c r="B28" s="61" t="s">
+      <c r="B28" s="33" t="s">
         <v>429</v>
       </c>
-      <c r="C28" s="61">
+      <c r="C28" s="33">
         <v>8719558935161</v>
       </c>
-      <c r="D28" s="61" t="s">
+      <c r="D28" s="33" t="s">
         <v>431</v>
       </c>
-      <c r="E28" s="61" t="s">
+      <c r="E28" s="33" t="s">
         <v>430</v>
       </c>
-      <c r="H28" s="61" t="s">
+      <c r="H28" s="33" t="s">
         <v>432</v>
       </c>
-      <c r="J28" s="61" t="s">
+      <c r="J28" s="33" t="s">
         <v>434</v>
       </c>
-      <c r="K28" s="61" t="s">
+      <c r="K28" s="88" t="s">
         <v>425</v>
       </c>
-      <c r="L28" s="61" t="s">
+      <c r="L28" s="88" t="s">
         <v>433</v>
       </c>
-      <c r="N28" s="61" t="s">
+      <c r="M28" s="88"/>
+      <c r="N28" s="88" t="s">
         <v>435</v>
       </c>
-      <c r="Z28" s="88" t="s">
+      <c r="O28" s="88"/>
+      <c r="P28" s="88"/>
+      <c r="Q28" s="88"/>
+      <c r="R28" s="88"/>
+      <c r="S28" s="88"/>
+      <c r="Z28" s="59" t="s">
         <v>436</v>
       </c>
-      <c r="AF28" s="61" t="s">
+      <c r="AF28" s="33" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="29" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A29" s="61">
+      <c r="A29" s="33">
         <v>98636312</v>
       </c>
-      <c r="B29" s="61" t="s">
+      <c r="B29" s="33" t="s">
         <v>438</v>
       </c>
-      <c r="C29" s="61">
+      <c r="C29" s="33">
         <v>8719558936502</v>
       </c>
-      <c r="D29" s="61" t="s">
+      <c r="D29" s="33" t="s">
         <v>439</v>
       </c>
-      <c r="E29" s="61" t="s">
+      <c r="E29" s="33" t="s">
         <v>430</v>
       </c>
-      <c r="H29" s="61" t="s">
+      <c r="H29" s="33" t="s">
         <v>440</v>
       </c>
-      <c r="J29" s="61" t="s">
+      <c r="J29" s="33" t="s">
         <v>442</v>
       </c>
-      <c r="K29" s="61" t="s">
+      <c r="K29" s="88" t="s">
         <v>425</v>
       </c>
-      <c r="L29" s="61" t="s">
+      <c r="L29" s="88" t="s">
         <v>441</v>
       </c>
-      <c r="N29" s="61" t="s">
+      <c r="M29" s="88"/>
+      <c r="N29" s="88" t="s">
         <v>250</v>
       </c>
-      <c r="Z29" s="88" t="s">
+      <c r="O29" s="88"/>
+      <c r="P29" s="88"/>
+      <c r="Q29" s="88"/>
+      <c r="R29" s="88"/>
+      <c r="S29" s="88"/>
+      <c r="Z29" s="59" t="s">
         <v>443</v>
       </c>
-      <c r="AF29" s="61" t="s">
+      <c r="AF29" s="33" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A30" s="61">
+      <c r="A30" s="33">
         <v>99218629</v>
       </c>
-      <c r="D30" s="61" t="s">
+      <c r="D30" s="33" t="s">
         <v>445</v>
       </c>
-      <c r="E30" s="61" t="s">
+      <c r="E30" s="33" t="s">
         <v>446</v>
       </c>
+      <c r="K30" s="88"/>
+      <c r="L30" s="88"/>
+      <c r="M30" s="88"/>
+      <c r="N30" s="88"/>
+      <c r="O30" s="88"/>
+      <c r="P30" s="88"/>
+      <c r="Q30" s="88"/>
+      <c r="R30" s="88"/>
+      <c r="S30" s="88"/>
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A31" s="61">
+      <c r="A31" s="33">
         <v>99218809</v>
       </c>
-      <c r="D31" s="61" t="s">
+      <c r="D31" s="33" t="s">
         <v>449</v>
       </c>
-      <c r="E31" s="61" t="s">
+      <c r="E31" s="33" t="s">
         <v>447</v>
       </c>
-      <c r="G31" s="61" t="s">
+      <c r="G31" s="33" t="s">
         <v>448</v>
       </c>
-      <c r="H31" s="61" t="s">
+      <c r="H31" s="33" t="s">
         <v>447</v>
       </c>
+      <c r="K31" s="88"/>
+      <c r="L31" s="88"/>
+      <c r="M31" s="88"/>
+      <c r="N31" s="88"/>
+      <c r="O31" s="88"/>
+      <c r="P31" s="88"/>
+      <c r="Q31" s="88"/>
+      <c r="R31" s="88"/>
+      <c r="S31" s="88"/>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A32" s="61">
+      <c r="A32" s="33">
         <v>99218810</v>
       </c>
-      <c r="D32" s="61" t="s">
+      <c r="D32" s="33" t="s">
         <v>450</v>
       </c>
-      <c r="E32" s="61" t="s">
+      <c r="E32" s="33" t="s">
         <v>447</v>
       </c>
-      <c r="G32" s="61" t="s">
+      <c r="G32" s="33" t="s">
         <v>448</v>
       </c>
-      <c r="H32" s="61" t="s">
+      <c r="H32" s="33" t="s">
         <v>447</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="61">
+      <c r="A33" s="33">
         <v>99218793</v>
       </c>
-      <c r="D33" s="61" t="s">
+      <c r="D33" s="33" t="s">
         <v>450</v>
       </c>
-      <c r="E33" s="61" t="s">
+      <c r="E33" s="33" t="s">
         <v>447</v>
       </c>
-      <c r="G33" s="61" t="s">
+      <c r="G33" s="33" t="s">
         <v>448</v>
       </c>
-      <c r="H33" s="61" t="s">
+      <c r="H33" s="33" t="s">
         <v>447</v>
       </c>
     </row>
@@ -3804,568 +3860,568 @@
   <dimension ref="A1:T25"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.140625" style="62" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" style="62" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" style="62" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" style="62" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="62" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.85546875" style="62" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" style="62" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" style="62" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.42578125" style="62" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" style="62" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" style="62" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.140625" style="62" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14" style="62" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="36.85546875" style="64" customWidth="1"/>
-    <col min="16" max="16" width="14" style="62" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.28515625" style="62" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="14.42578125" style="62"/>
+    <col min="1" max="1" width="14.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14" style="34" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="36.85546875" style="36" customWidth="1"/>
+    <col min="16" max="16" width="14" style="34" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.28515625" style="34" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="14.42578125" style="34"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="59" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+    <row r="1" spans="1:20" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="31" t="s">
         <v>253</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="31" t="s">
         <v>254</v>
       </c>
-      <c r="C1" s="60" t="s">
+      <c r="C1" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="D1" s="60" t="s">
+      <c r="D1" s="32" t="s">
         <v>256</v>
       </c>
-      <c r="E1" s="60" t="s">
+      <c r="E1" s="32" t="s">
         <v>257</v>
       </c>
-      <c r="F1" s="60" t="s">
+      <c r="F1" s="32" t="s">
         <v>258</v>
       </c>
-      <c r="G1" s="60" t="s">
+      <c r="G1" s="32" t="s">
         <v>259</v>
       </c>
-      <c r="H1" s="59" t="s">
+      <c r="H1" s="31" t="s">
         <v>260</v>
       </c>
-      <c r="I1" s="59" t="s">
+      <c r="I1" s="31" t="s">
         <v>261</v>
       </c>
-      <c r="J1" s="59" t="s">
+      <c r="J1" s="31" t="s">
         <v>262</v>
       </c>
-      <c r="K1" s="59" t="s">
+      <c r="K1" s="31" t="s">
         <v>263</v>
       </c>
-      <c r="L1" s="59" t="s">
+      <c r="L1" s="31" t="s">
         <v>264</v>
       </c>
-      <c r="M1" s="59" t="s">
+      <c r="M1" s="31" t="s">
         <v>265</v>
       </c>
-      <c r="N1" s="59" t="s">
+      <c r="N1" s="31" t="s">
         <v>266</v>
       </c>
-      <c r="O1" s="59" t="s">
+      <c r="O1" s="31" t="s">
         <v>267</v>
       </c>
-      <c r="P1" s="59" t="s">
+      <c r="P1" s="31" t="s">
         <v>268</v>
       </c>
-      <c r="Q1" s="59" t="s">
+      <c r="Q1" s="31" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="135" x14ac:dyDescent="0.25">
-      <c r="A2" s="30">
+      <c r="A2" s="28">
         <v>5401209028218</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="4">
         <v>88884444</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="63" t="s">
+      <c r="D2" s="35" t="s">
         <v>270</v>
       </c>
-      <c r="E2" s="63" t="s">
+      <c r="E2" s="35" t="s">
         <v>249</v>
       </c>
-      <c r="F2" s="63" t="s">
+      <c r="F2" s="35" t="s">
         <v>277</v>
       </c>
-      <c r="G2" s="63" t="s">
+      <c r="G2" s="35" t="s">
         <v>276</v>
       </c>
-      <c r="H2" s="62" t="s">
+      <c r="H2" s="34" t="s">
         <v>271</v>
       </c>
-      <c r="I2" s="62" t="s">
+      <c r="I2" s="34" t="s">
         <v>272</v>
       </c>
-      <c r="J2" s="62" t="s">
+      <c r="J2" s="34" t="s">
         <v>281</v>
       </c>
-      <c r="K2" s="62" t="s">
+      <c r="K2" s="34" t="s">
         <v>280</v>
       </c>
-      <c r="L2" s="62" t="s">
+      <c r="L2" s="34" t="s">
         <v>283</v>
       </c>
-      <c r="M2" s="62" t="s">
+      <c r="M2" s="34" t="s">
         <v>284</v>
       </c>
-      <c r="N2" s="64" t="s">
+      <c r="N2" s="36" t="s">
         <v>287</v>
       </c>
-      <c r="O2" s="64" t="s">
+      <c r="O2" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="P2" s="62" t="s">
+      <c r="P2" s="34" t="s">
         <v>273</v>
       </c>
-      <c r="Q2" s="62" t="s">
+      <c r="Q2" s="34" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="135" x14ac:dyDescent="0.25">
-      <c r="A3" s="30">
+      <c r="A3" s="28">
         <v>5401209028219</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="4">
         <v>88884445</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="D3" s="63" t="s">
+      <c r="D3" s="35" t="s">
         <v>270</v>
       </c>
-      <c r="E3" s="63" t="s">
+      <c r="E3" s="35" t="s">
         <v>249</v>
       </c>
-      <c r="F3" s="63" t="s">
+      <c r="F3" s="35" t="s">
         <v>278</v>
       </c>
-      <c r="G3" s="63" t="s">
+      <c r="G3" s="35" t="s">
         <v>275</v>
       </c>
-      <c r="H3" s="62" t="s">
+      <c r="H3" s="34" t="s">
         <v>271</v>
       </c>
-      <c r="I3" s="62" t="s">
+      <c r="I3" s="34" t="s">
         <v>279</v>
       </c>
-      <c r="J3" s="62" t="s">
+      <c r="J3" s="34" t="s">
         <v>281</v>
       </c>
-      <c r="K3" s="62" t="s">
+      <c r="K3" s="34" t="s">
         <v>280</v>
       </c>
-      <c r="L3" s="62" t="s">
+      <c r="L3" s="34" t="s">
         <v>282</v>
       </c>
-      <c r="M3" s="62" t="s">
+      <c r="M3" s="34" t="s">
         <v>285</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="36" t="s">
         <v>286</v>
       </c>
-      <c r="O3" s="64" t="s">
+      <c r="O3" s="36" t="s">
         <v>289</v>
       </c>
-      <c r="P3" s="62" t="s">
+      <c r="P3" s="34" t="s">
         <v>273</v>
       </c>
-      <c r="Q3" s="62" t="s">
+      <c r="Q3" s="34" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="66"/>
-      <c r="B5" s="65"/>
-      <c r="C5" s="62"/>
-      <c r="D5" s="62"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
-      <c r="I5" s="65"/>
-      <c r="J5" s="65"/>
-      <c r="K5" s="65"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="65"/>
-      <c r="R5" s="65"/>
+      <c r="A5" s="38"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="R5" s="37"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A6" s="65"/>
+      <c r="A6" s="37"/>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="41" t="s">
         <v>303</v>
       </c>
-      <c r="B8" s="68">
+      <c r="B8" s="40">
         <v>90861025</v>
       </c>
-      <c r="H8" s="68" t="s">
+      <c r="H8" s="40" t="s">
         <v>309</v>
       </c>
-      <c r="I8" s="68" t="s">
+      <c r="I8" s="40" t="s">
         <v>310</v>
       </c>
-      <c r="N8" s="68" t="s">
+      <c r="N8" s="40" t="s">
         <v>305</v>
       </c>
-      <c r="O8" s="68" t="s">
+      <c r="O8" s="40" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A9" s="68"/>
-      <c r="B9" s="68"/>
-      <c r="C9" s="68"/>
-      <c r="D9" s="69"/>
-      <c r="E9" s="68"/>
-      <c r="F9" s="70"/>
-      <c r="G9" s="68"/>
-      <c r="H9" s="68"/>
-      <c r="I9" s="68"/>
-      <c r="J9" s="68"/>
-      <c r="K9" s="68"/>
-      <c r="L9" s="68"/>
-      <c r="M9" s="68"/>
-      <c r="N9" s="68"/>
-      <c r="O9" s="68"/>
-      <c r="P9" s="68"/>
-      <c r="Q9" s="68"/>
-      <c r="R9" s="68"/>
-      <c r="S9" s="68"/>
-      <c r="T9" s="68"/>
+      <c r="A9" s="40"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="40"/>
+      <c r="H9" s="40"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="40"/>
+      <c r="K9" s="40"/>
+      <c r="L9" s="40"/>
+      <c r="M9" s="40"/>
+      <c r="N9" s="40"/>
+      <c r="O9" s="40"/>
+      <c r="P9" s="40"/>
+      <c r="Q9" s="40"/>
+      <c r="R9" s="40"/>
+      <c r="S9" s="40"/>
+      <c r="T9" s="40"/>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A10" s="68"/>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="69"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="70"/>
-      <c r="G10" s="68"/>
-      <c r="H10" s="68"/>
-      <c r="I10" s="68"/>
-      <c r="J10" s="68"/>
-      <c r="K10" s="68"/>
-      <c r="L10" s="68"/>
-      <c r="M10" s="68"/>
-      <c r="N10" s="68"/>
-      <c r="O10" s="68"/>
-      <c r="P10" s="68"/>
-      <c r="Q10" s="68"/>
-      <c r="R10" s="68"/>
-      <c r="S10" s="68"/>
-      <c r="T10" s="68"/>
+      <c r="A10" s="40"/>
+      <c r="B10" s="40"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="40"/>
+      <c r="I10" s="40"/>
+      <c r="J10" s="40"/>
+      <c r="K10" s="40"/>
+      <c r="L10" s="40"/>
+      <c r="M10" s="40"/>
+      <c r="N10" s="40"/>
+      <c r="O10" s="40"/>
+      <c r="P10" s="40"/>
+      <c r="Q10" s="40"/>
+      <c r="R10" s="40"/>
+      <c r="S10" s="40"/>
+      <c r="T10" s="40"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A11" s="68"/>
-      <c r="B11" s="68"/>
-      <c r="C11" s="68"/>
-      <c r="D11" s="69"/>
-      <c r="E11" s="68"/>
-      <c r="F11" s="70"/>
-      <c r="G11" s="68"/>
-      <c r="H11" s="68"/>
-      <c r="I11" s="68"/>
-      <c r="J11" s="68"/>
-      <c r="K11" s="68"/>
-      <c r="L11" s="68"/>
-      <c r="M11" s="68"/>
-      <c r="N11" s="68"/>
-      <c r="O11" s="68"/>
-      <c r="P11" s="68"/>
-      <c r="Q11" s="68"/>
-      <c r="R11" s="68"/>
-      <c r="S11" s="68"/>
-      <c r="T11" s="68"/>
+      <c r="A11" s="40"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="40"/>
+      <c r="M11" s="40"/>
+      <c r="N11" s="40"/>
+      <c r="O11" s="40"/>
+      <c r="P11" s="40"/>
+      <c r="Q11" s="40"/>
+      <c r="R11" s="40"/>
+      <c r="S11" s="40"/>
+      <c r="T11" s="40"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A12" s="68"/>
-      <c r="B12" s="68"/>
-      <c r="C12" s="68"/>
-      <c r="D12" s="69"/>
-      <c r="E12" s="68"/>
-      <c r="F12" s="70"/>
-      <c r="G12" s="68"/>
-      <c r="H12" s="68"/>
-      <c r="I12" s="68"/>
-      <c r="J12" s="68"/>
-      <c r="K12" s="68"/>
-      <c r="L12" s="68"/>
-      <c r="M12" s="68"/>
-      <c r="N12" s="68"/>
-      <c r="O12" s="68"/>
-      <c r="P12" s="68"/>
-      <c r="Q12" s="68"/>
-      <c r="R12" s="68"/>
-      <c r="S12" s="68"/>
-      <c r="T12" s="68"/>
+      <c r="A12" s="40"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="40"/>
+      <c r="K12" s="40"/>
+      <c r="L12" s="40"/>
+      <c r="M12" s="40"/>
+      <c r="N12" s="40"/>
+      <c r="O12" s="40"/>
+      <c r="P12" s="40"/>
+      <c r="Q12" s="40"/>
+      <c r="R12" s="40"/>
+      <c r="S12" s="40"/>
+      <c r="T12" s="40"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13" s="68"/>
-      <c r="B13" s="68"/>
-      <c r="C13" s="68"/>
-      <c r="D13" s="69"/>
-      <c r="E13" s="68"/>
-      <c r="F13" s="70"/>
-      <c r="G13" s="68"/>
-      <c r="H13" s="68"/>
-      <c r="I13" s="68"/>
-      <c r="J13" s="68"/>
-      <c r="K13" s="68"/>
-      <c r="L13" s="68"/>
-      <c r="M13" s="68"/>
-      <c r="N13" s="68"/>
-      <c r="O13" s="68"/>
-      <c r="P13" s="68"/>
-      <c r="Q13" s="68"/>
-      <c r="R13" s="68"/>
-      <c r="S13" s="68"/>
-      <c r="T13" s="68"/>
+      <c r="A13" s="40"/>
+      <c r="B13" s="40"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="40"/>
+      <c r="K13" s="40"/>
+      <c r="L13" s="40"/>
+      <c r="M13" s="40"/>
+      <c r="N13" s="40"/>
+      <c r="O13" s="40"/>
+      <c r="P13" s="40"/>
+      <c r="Q13" s="40"/>
+      <c r="R13" s="40"/>
+      <c r="S13" s="40"/>
+      <c r="T13" s="40"/>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A14" s="68"/>
-      <c r="B14" s="68"/>
-      <c r="C14" s="68"/>
-      <c r="D14" s="69"/>
-      <c r="E14" s="68"/>
-      <c r="F14" s="70"/>
-      <c r="G14" s="68"/>
-      <c r="H14" s="68"/>
-      <c r="I14" s="68"/>
-      <c r="J14" s="68"/>
-      <c r="K14" s="68"/>
-      <c r="L14" s="68"/>
-      <c r="M14" s="68"/>
-      <c r="N14" s="68"/>
-      <c r="O14" s="68"/>
-      <c r="P14" s="68"/>
-      <c r="Q14" s="68"/>
-      <c r="R14" s="68"/>
-      <c r="S14" s="68"/>
-      <c r="T14" s="68"/>
+      <c r="A14" s="40"/>
+      <c r="B14" s="40"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
+      <c r="J14" s="40"/>
+      <c r="K14" s="40"/>
+      <c r="L14" s="40"/>
+      <c r="M14" s="40"/>
+      <c r="N14" s="40"/>
+      <c r="O14" s="40"/>
+      <c r="P14" s="40"/>
+      <c r="Q14" s="40"/>
+      <c r="R14" s="40"/>
+      <c r="S14" s="40"/>
+      <c r="T14" s="40"/>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A15" s="68"/>
-      <c r="B15" s="68"/>
-      <c r="C15" s="68"/>
-      <c r="D15" s="69"/>
-      <c r="E15" s="68"/>
-      <c r="F15" s="70"/>
-      <c r="G15" s="68"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="68"/>
-      <c r="J15" s="68"/>
-      <c r="K15" s="68"/>
-      <c r="L15" s="68"/>
-      <c r="M15" s="68"/>
-      <c r="N15" s="68"/>
-      <c r="O15" s="68"/>
-      <c r="P15" s="68"/>
-      <c r="Q15" s="68"/>
-      <c r="R15" s="68"/>
-      <c r="S15" s="68"/>
-      <c r="T15" s="68"/>
+      <c r="A15" s="40"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="40"/>
+      <c r="K15" s="40"/>
+      <c r="L15" s="40"/>
+      <c r="M15" s="40"/>
+      <c r="N15" s="40"/>
+      <c r="O15" s="40"/>
+      <c r="P15" s="40"/>
+      <c r="Q15" s="40"/>
+      <c r="R15" s="40"/>
+      <c r="S15" s="40"/>
+      <c r="T15" s="40"/>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A16" s="68"/>
-      <c r="B16" s="68"/>
-      <c r="C16" s="68"/>
-      <c r="D16" s="69"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="68"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="68"/>
-      <c r="J16" s="68"/>
-      <c r="K16" s="68"/>
-      <c r="L16" s="68"/>
-      <c r="M16" s="68"/>
-      <c r="N16" s="68"/>
-      <c r="O16" s="68"/>
-      <c r="P16" s="68"/>
-      <c r="Q16" s="68"/>
-      <c r="R16" s="68"/>
-      <c r="S16" s="68"/>
-      <c r="T16" s="68"/>
+      <c r="A16" s="40"/>
+      <c r="B16" s="40"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="40"/>
+      <c r="K16" s="40"/>
+      <c r="L16" s="40"/>
+      <c r="M16" s="40"/>
+      <c r="N16" s="40"/>
+      <c r="O16" s="40"/>
+      <c r="P16" s="40"/>
+      <c r="Q16" s="40"/>
+      <c r="R16" s="40"/>
+      <c r="S16" s="40"/>
+      <c r="T16" s="40"/>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A17" s="68"/>
-      <c r="B17" s="68"/>
-      <c r="C17" s="68"/>
-      <c r="D17" s="69"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="70"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="68"/>
-      <c r="J17" s="68"/>
-      <c r="K17" s="68"/>
-      <c r="L17" s="68"/>
-      <c r="M17" s="68"/>
-      <c r="N17" s="68"/>
-      <c r="O17" s="68"/>
-      <c r="P17" s="68"/>
-      <c r="Q17" s="68"/>
-      <c r="R17" s="68"/>
-      <c r="S17" s="68"/>
-      <c r="T17" s="68"/>
+      <c r="A17" s="40"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="40"/>
+      <c r="K17" s="40"/>
+      <c r="L17" s="40"/>
+      <c r="M17" s="40"/>
+      <c r="N17" s="40"/>
+      <c r="O17" s="40"/>
+      <c r="P17" s="40"/>
+      <c r="Q17" s="40"/>
+      <c r="R17" s="40"/>
+      <c r="S17" s="40"/>
+      <c r="T17" s="40"/>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A18" s="68"/>
-      <c r="B18" s="68"/>
-      <c r="C18" s="68"/>
-      <c r="D18" s="69"/>
-      <c r="E18" s="68"/>
-      <c r="F18" s="70"/>
-      <c r="G18" s="68"/>
-      <c r="H18" s="68"/>
-      <c r="I18" s="68"/>
-      <c r="J18" s="68"/>
-      <c r="K18" s="68"/>
-      <c r="L18" s="68"/>
-      <c r="M18" s="68"/>
-      <c r="N18" s="68"/>
-      <c r="O18" s="68"/>
-      <c r="P18" s="68"/>
-      <c r="Q18" s="68"/>
-      <c r="R18" s="68"/>
-      <c r="S18" s="68"/>
-      <c r="T18" s="68"/>
+      <c r="A18" s="40"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="40"/>
+      <c r="N18" s="40"/>
+      <c r="O18" s="40"/>
+      <c r="P18" s="40"/>
+      <c r="Q18" s="40"/>
+      <c r="R18" s="40"/>
+      <c r="S18" s="40"/>
+      <c r="T18" s="40"/>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A19" s="68"/>
-      <c r="B19" s="68"/>
-      <c r="C19" s="68"/>
-      <c r="D19" s="69"/>
-      <c r="E19" s="68"/>
-      <c r="F19" s="70"/>
-      <c r="G19" s="68"/>
-      <c r="H19" s="68"/>
-      <c r="I19" s="68"/>
-      <c r="J19" s="68"/>
-      <c r="K19" s="68"/>
-      <c r="L19" s="68"/>
-      <c r="M19" s="68"/>
-      <c r="N19" s="68"/>
-      <c r="O19" s="68"/>
-      <c r="P19" s="68"/>
-      <c r="Q19" s="68"/>
-      <c r="R19" s="68"/>
-      <c r="S19" s="68"/>
-      <c r="T19" s="68"/>
+      <c r="A19" s="40"/>
+      <c r="B19" s="40"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="40"/>
+      <c r="H19" s="40"/>
+      <c r="I19" s="40"/>
+      <c r="J19" s="40"/>
+      <c r="K19" s="40"/>
+      <c r="L19" s="40"/>
+      <c r="M19" s="40"/>
+      <c r="N19" s="40"/>
+      <c r="O19" s="40"/>
+      <c r="P19" s="40"/>
+      <c r="Q19" s="40"/>
+      <c r="R19" s="40"/>
+      <c r="S19" s="40"/>
+      <c r="T19" s="40"/>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A20" s="68"/>
-      <c r="B20" s="68"/>
-      <c r="C20" s="68"/>
-      <c r="D20" s="69"/>
-      <c r="E20" s="68"/>
-      <c r="F20" s="70"/>
-      <c r="G20" s="68"/>
-      <c r="H20" s="68"/>
-      <c r="I20" s="68"/>
-      <c r="J20" s="68"/>
-      <c r="K20" s="68"/>
-      <c r="L20" s="68"/>
-      <c r="M20" s="68"/>
-      <c r="N20" s="68"/>
-      <c r="O20" s="68"/>
-      <c r="P20" s="68"/>
-      <c r="Q20" s="68"/>
-      <c r="R20" s="68"/>
-      <c r="S20" s="68"/>
-      <c r="T20" s="68"/>
+      <c r="A20" s="40"/>
+      <c r="B20" s="40"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="40"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="40"/>
+      <c r="J20" s="40"/>
+      <c r="K20" s="40"/>
+      <c r="L20" s="40"/>
+      <c r="M20" s="40"/>
+      <c r="N20" s="40"/>
+      <c r="O20" s="40"/>
+      <c r="P20" s="40"/>
+      <c r="Q20" s="40"/>
+      <c r="R20" s="40"/>
+      <c r="S20" s="40"/>
+      <c r="T20" s="40"/>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A21" s="68"/>
-      <c r="B21" s="68"/>
-      <c r="C21" s="68"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="68"/>
-      <c r="F21" s="70"/>
-      <c r="G21" s="68"/>
-      <c r="H21" s="68"/>
-      <c r="I21" s="68"/>
-      <c r="J21" s="68"/>
-      <c r="K21" s="68"/>
-      <c r="L21" s="68"/>
-      <c r="M21" s="68"/>
-      <c r="N21" s="68"/>
-      <c r="O21" s="68"/>
-      <c r="P21" s="68"/>
-      <c r="Q21" s="68"/>
-      <c r="R21" s="68"/>
-      <c r="S21" s="68"/>
-      <c r="T21" s="68"/>
+      <c r="A21" s="40"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="40"/>
+      <c r="M21" s="40"/>
+      <c r="N21" s="40"/>
+      <c r="O21" s="40"/>
+      <c r="P21" s="40"/>
+      <c r="Q21" s="40"/>
+      <c r="R21" s="40"/>
+      <c r="S21" s="40"/>
+      <c r="T21" s="40"/>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A22" s="68"/>
-      <c r="B22" s="68"/>
-      <c r="C22" s="68"/>
-      <c r="D22" s="69"/>
-      <c r="E22" s="68"/>
-      <c r="F22" s="70"/>
-      <c r="G22" s="68"/>
-      <c r="H22" s="68"/>
-      <c r="I22" s="68"/>
-      <c r="J22" s="68"/>
-      <c r="K22" s="68"/>
-      <c r="L22" s="68"/>
-      <c r="M22" s="68"/>
+      <c r="A22" s="40"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="40"/>
+      <c r="J22" s="40"/>
+      <c r="K22" s="40"/>
+      <c r="L22" s="40"/>
+      <c r="M22" s="40"/>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A23" s="68"/>
-      <c r="B23" s="68"/>
-      <c r="C23" s="68"/>
-      <c r="D23" s="69"/>
-      <c r="E23" s="68"/>
-      <c r="F23" s="70"/>
-      <c r="G23" s="68"/>
-      <c r="H23" s="68"/>
-      <c r="I23" s="68"/>
-      <c r="J23" s="68"/>
-      <c r="K23" s="68"/>
-      <c r="L23" s="68"/>
-      <c r="M23" s="68"/>
+      <c r="A23" s="40"/>
+      <c r="B23" s="40"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="40"/>
+      <c r="J23" s="40"/>
+      <c r="K23" s="40"/>
+      <c r="L23" s="40"/>
+      <c r="M23" s="40"/>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A24" s="68"/>
-      <c r="B24" s="68"/>
-      <c r="C24" s="68"/>
-      <c r="D24" s="69"/>
-      <c r="E24" s="68"/>
-      <c r="F24" s="70"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
-      <c r="J24" s="68"/>
-      <c r="K24" s="68"/>
-      <c r="L24" s="68"/>
-      <c r="M24" s="68"/>
+      <c r="A24" s="40"/>
+      <c r="B24" s="40"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
+      <c r="J24" s="40"/>
+      <c r="K24" s="40"/>
+      <c r="L24" s="40"/>
+      <c r="M24" s="40"/>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A25" s="68"/>
-      <c r="B25" s="68"/>
-      <c r="C25" s="68"/>
-      <c r="D25" s="69"/>
-      <c r="E25" s="68"/>
-      <c r="F25" s="70"/>
-      <c r="G25" s="68"/>
-      <c r="H25" s="68"/>
-      <c r="I25" s="68"/>
-      <c r="J25" s="68"/>
-      <c r="K25" s="68"/>
-      <c r="L25" s="68"/>
-      <c r="M25" s="68"/>
+      <c r="A25" s="40"/>
+      <c r="B25" s="40"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="40"/>
+      <c r="J25" s="40"/>
+      <c r="K25" s="40"/>
+      <c r="L25" s="40"/>
+      <c r="M25" s="40"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5386,395 +5442,395 @@
   <dimension ref="A1:R46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="18.42578125" style="6" customWidth="1"/>
-    <col min="4" max="15" width="16.140625" style="6" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="6"/>
+    <col min="1" max="3" width="18.42578125" style="4" customWidth="1"/>
+    <col min="4" max="15" width="16.140625" style="4" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5"/>
-      <c r="B1" s="5"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="33" t="s">
+      <c r="A1" s="64"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="68" t="s">
         <v>216</v>
       </c>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="36" t="s">
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="71" t="s">
         <v>217</v>
       </c>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="38"/>
-      <c r="P1" s="39" t="s">
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="74" t="s">
         <v>216</v>
       </c>
-      <c r="Q1" s="40"/>
-      <c r="R1" s="8"/>
+      <c r="Q1" s="75"/>
+      <c r="R1" s="6"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="41" t="s">
+      <c r="A2" s="64"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="76" t="s">
         <v>218</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="44" t="s">
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="79" t="s">
         <v>219</v>
       </c>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="47" t="s">
+      <c r="K2" s="80"/>
+      <c r="L2" s="80"/>
+      <c r="M2" s="80"/>
+      <c r="N2" s="80"/>
+      <c r="O2" s="81"/>
+      <c r="P2" s="82" t="s">
         <v>220</v>
       </c>
-      <c r="Q2" s="48"/>
-      <c r="R2" s="7"/>
+      <c r="Q2" s="83"/>
+      <c r="R2" s="5"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="49" t="s">
+      <c r="A3" s="64"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="84" t="s">
         <v>221</v>
       </c>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="51" t="s">
+      <c r="E3" s="85"/>
+      <c r="F3" s="85"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="86" t="s">
         <v>222</v>
       </c>
-      <c r="I3" s="52"/>
-      <c r="J3" s="49" t="s">
+      <c r="I3" s="87"/>
+      <c r="J3" s="84" t="s">
         <v>223</v>
       </c>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="52"/>
-      <c r="P3" s="53" t="s">
+      <c r="K3" s="85"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="85"/>
+      <c r="O3" s="87"/>
+      <c r="P3" s="60" t="s">
         <v>224</v>
       </c>
-      <c r="Q3" s="54" t="s">
+      <c r="Q3" s="62" t="s">
         <v>225</v>
       </c>
-      <c r="R3" s="7"/>
+      <c r="R3" s="5"/>
     </row>
     <row r="4" spans="1:18" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="55"/>
-      <c r="B4" s="55"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="11" t="s">
+      <c r="A4" s="66"/>
+      <c r="B4" s="66"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="K4" s="18" t="s">
+      <c r="K4" s="16" t="s">
         <v>233</v>
       </c>
-      <c r="L4" s="18" t="s">
+      <c r="L4" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="M4" s="19" t="s">
+      <c r="M4" s="17" t="s">
         <v>235</v>
       </c>
-      <c r="N4" s="19" t="s">
+      <c r="N4" s="17" t="s">
         <v>236</v>
       </c>
-      <c r="O4" s="20" t="s">
+      <c r="O4" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="P4" s="57"/>
-      <c r="Q4" s="58"/>
-      <c r="R4" s="7"/>
+      <c r="P4" s="61"/>
+      <c r="Q4" s="63"/>
+      <c r="R4" s="5"/>
     </row>
     <row r="5" spans="1:18" ht="240.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="G5" s="22" t="s">
+      <c r="G5" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="I5" s="24" t="s">
+      <c r="I5" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="J5" s="25" t="s">
+      <c r="J5" s="23" t="s">
         <v>245</v>
       </c>
-      <c r="K5" s="26" t="s">
+      <c r="K5" s="24" t="s">
         <v>245</v>
       </c>
-      <c r="L5" s="26" t="s">
+      <c r="L5" s="24" t="s">
         <v>245</v>
       </c>
-      <c r="M5" s="26" t="s">
+      <c r="M5" s="24" t="s">
         <v>245</v>
       </c>
-      <c r="N5" s="26" t="s">
+      <c r="N5" s="24" t="s">
         <v>245</v>
       </c>
-      <c r="O5" s="27" t="s">
+      <c r="O5" s="25" t="s">
         <v>245</v>
       </c>
-      <c r="P5" s="28" t="s">
+      <c r="P5" s="26" t="s">
         <v>246</v>
       </c>
-      <c r="Q5" s="29" t="s">
+      <c r="Q5" s="27" t="s">
         <v>247</v>
       </c>
-      <c r="R5" s="7"/>
+      <c r="R5" s="5"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="31"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
+      <c r="A6" s="29"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="31"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="31"/>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
+      <c r="A8" s="29"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="31"/>
-      <c r="B9" s="32"/>
-      <c r="C9" s="32"/>
+      <c r="A9" s="29"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A10" s="31"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
+      <c r="A10" s="29"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="31"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
+      <c r="A11" s="29"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="31"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
+      <c r="A12" s="29"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="31"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
+      <c r="A13" s="29"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" s="31"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
+      <c r="A14" s="29"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="31"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
+      <c r="A15" s="29"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="31"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
+      <c r="A16" s="29"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="31"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
+      <c r="A17" s="29"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="31"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
+      <c r="A18" s="29"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="31"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
+      <c r="A19" s="29"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="31"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
+      <c r="A20" s="29"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="31"/>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
+      <c r="A21" s="29"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="31"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="31"/>
-      <c r="B23" s="32"/>
-      <c r="C23" s="32"/>
+      <c r="A23" s="29"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="31"/>
-      <c r="B24" s="32"/>
-      <c r="C24" s="32"/>
+      <c r="A24" s="29"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="31"/>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
+      <c r="A25" s="29"/>
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="31"/>
-      <c r="B26" s="32"/>
-      <c r="C26" s="32"/>
+      <c r="A26" s="29"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="30"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="31"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
+      <c r="A27" s="29"/>
+      <c r="B27" s="30"/>
+      <c r="C27" s="30"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="31"/>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
+      <c r="A28" s="29"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="30"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="31"/>
-      <c r="B29" s="32"/>
-      <c r="C29" s="32"/>
+      <c r="A29" s="29"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="31"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
+      <c r="A30" s="29"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="30"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="31"/>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
+      <c r="A31" s="29"/>
+      <c r="B31" s="30"/>
+      <c r="C31" s="30"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="31"/>
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
+      <c r="A32" s="29"/>
+      <c r="B32" s="30"/>
+      <c r="C32" s="30"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="31"/>
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
+      <c r="A33" s="29"/>
+      <c r="B33" s="30"/>
+      <c r="C33" s="30"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="31"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
+      <c r="A34" s="29"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="31"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
+      <c r="A35" s="29"/>
+      <c r="B35" s="30"/>
+      <c r="C35" s="30"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="31"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
+      <c r="A36" s="29"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="30"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="31"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
+      <c r="A37" s="29"/>
+      <c r="B37" s="30"/>
+      <c r="C37" s="30"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="31"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
+      <c r="A38" s="29"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="30"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="31"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
+      <c r="A39" s="29"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="30"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="31"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
+      <c r="A40" s="29"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="30"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="31"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
+      <c r="A41" s="29"/>
+      <c r="B41" s="30"/>
+      <c r="C41" s="30"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="31"/>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
+      <c r="A42" s="29"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="30"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="31"/>
-      <c r="B43" s="32"/>
-      <c r="C43" s="32"/>
+      <c r="A43" s="29"/>
+      <c r="B43" s="30"/>
+      <c r="C43" s="30"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="31"/>
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
+      <c r="A44" s="29"/>
+      <c r="B44" s="30"/>
+      <c r="C44" s="30"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="31"/>
-      <c r="B45" s="32"/>
-      <c r="C45" s="32"/>
+      <c r="A45" s="29"/>
+      <c r="B45" s="30"/>
+      <c r="C45" s="30"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="31"/>
-      <c r="B46" s="32"/>
-      <c r="C46" s="32"/>
+      <c r="A46" s="29"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
CiMini additions to expand matching edge cases, ordering, phenotypes, transformation handling
</commit_message>
<xml_diff>
--- a/test/datasets/CiMini/Brackets-Complete.xlsx
+++ b/test/datasets/CiMini/Brackets-Complete.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="484">
   <si>
     <t>familyID</t>
   </si>
@@ -1767,6 +1767,105 @@
   </si>
   <si>
     <t>White socks - tennis</t>
+  </si>
+  <si>
+    <t>6318-5274</t>
+  </si>
+  <si>
+    <t>6318-7392</t>
+  </si>
+  <si>
+    <t>Grey</t>
+  </si>
+  <si>
+    <t>6417-6318</t>
+  </si>
+  <si>
+    <t>Navy</t>
+  </si>
+  <si>
+    <t>6318-4903</t>
+  </si>
+  <si>
+    <t>SHIRT</t>
+  </si>
+  <si>
+    <t>White</t>
+  </si>
+  <si>
+    <t>5274-5836</t>
+  </si>
+  <si>
+    <t>Beige</t>
+  </si>
+  <si>
+    <t>7215-5274</t>
+  </si>
+  <si>
+    <t>PANTS</t>
+  </si>
+  <si>
+    <t>3820-771</t>
+  </si>
+  <si>
+    <t>3820-772</t>
+  </si>
+  <si>
+    <t>A charcoal, grey-toned wrap for cool evenings</t>
+  </si>
+  <si>
+    <t>4560-410</t>
+  </si>
+  <si>
+    <t>Hoodie</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>5730-330</t>
+  </si>
+  <si>
+    <t>Blouse</t>
+  </si>
+  <si>
+    <t>6840-901</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>7950-220</t>
+  </si>
+  <si>
+    <t>Indigo Blue</t>
+  </si>
+  <si>
+    <t>3061-115</t>
+  </si>
+  <si>
+    <t>Denim Jacket</t>
+  </si>
+  <si>
+    <t>3061-116</t>
+  </si>
+  <si>
+    <t>Denim Vest</t>
+  </si>
+  <si>
+    <t>3061-117</t>
+  </si>
+  <si>
+    <t>Denim Shirt</t>
+  </si>
+  <si>
+    <t>4172-500</t>
+  </si>
+  <si>
+    <t>Sweater</t>
+  </si>
+  <si>
+    <t>5283-410</t>
   </si>
 </sst>
 </file>
@@ -2384,6 +2483,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2460,7 +2560,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2793,7 +2892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AF33"/>
+  <dimension ref="A1:AF50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" style="33" customWidth="1"/>
@@ -3559,15 +3658,15 @@
       <c r="E24" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="K24" s="88"/>
-      <c r="L24" s="88"/>
-      <c r="M24" s="88"/>
-      <c r="N24" s="88"/>
-      <c r="O24" s="88"/>
-      <c r="P24" s="88"/>
-      <c r="Q24" s="88"/>
-      <c r="R24" s="88"/>
-      <c r="S24" s="88"/>
+      <c r="K24" s="60"/>
+      <c r="L24" s="60"/>
+      <c r="M24" s="60"/>
+      <c r="N24" s="60"/>
+      <c r="O24" s="60"/>
+      <c r="P24" s="60"/>
+      <c r="Q24" s="60"/>
+      <c r="R24" s="60"/>
+      <c r="S24" s="60"/>
     </row>
     <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" s="33">
@@ -3588,17 +3687,17 @@
       <c r="H25" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="K25" s="88"/>
-      <c r="L25" s="88"/>
-      <c r="M25" s="88"/>
-      <c r="N25" s="88" t="s">
+      <c r="K25" s="60"/>
+      <c r="L25" s="60"/>
+      <c r="M25" s="60"/>
+      <c r="N25" s="60" t="s">
         <v>413</v>
       </c>
-      <c r="O25" s="88"/>
-      <c r="P25" s="88"/>
-      <c r="Q25" s="88"/>
-      <c r="R25" s="88"/>
-      <c r="S25" s="88"/>
+      <c r="O25" s="60"/>
+      <c r="P25" s="60"/>
+      <c r="Q25" s="60"/>
+      <c r="R25" s="60"/>
+      <c r="S25" s="60"/>
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" s="52">
@@ -3620,15 +3719,15 @@
       <c r="H26" s="33" t="s">
         <v>418</v>
       </c>
-      <c r="K26" s="88"/>
-      <c r="L26" s="88"/>
-      <c r="M26" s="88"/>
-      <c r="N26" s="88"/>
-      <c r="O26" s="88"/>
-      <c r="P26" s="88"/>
-      <c r="Q26" s="88"/>
-      <c r="R26" s="88"/>
-      <c r="S26" s="88"/>
+      <c r="K26" s="60"/>
+      <c r="L26" s="60"/>
+      <c r="M26" s="60"/>
+      <c r="N26" s="60"/>
+      <c r="O26" s="60"/>
+      <c r="P26" s="60"/>
+      <c r="Q26" s="60"/>
+      <c r="R26" s="60"/>
+      <c r="S26" s="60"/>
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" s="33">
@@ -3652,21 +3751,21 @@
       <c r="J27" s="33" t="s">
         <v>424</v>
       </c>
-      <c r="K27" s="88" t="s">
+      <c r="K27" s="60" t="s">
         <v>425</v>
       </c>
-      <c r="L27" s="88" t="s">
+      <c r="L27" s="60" t="s">
         <v>423</v>
       </c>
-      <c r="M27" s="88"/>
-      <c r="N27" s="88" t="s">
+      <c r="M27" s="60"/>
+      <c r="N27" s="60" t="s">
         <v>426</v>
       </c>
-      <c r="O27" s="88"/>
-      <c r="P27" s="88"/>
-      <c r="Q27" s="88"/>
-      <c r="R27" s="88"/>
-      <c r="S27" s="88"/>
+      <c r="O27" s="60"/>
+      <c r="P27" s="60"/>
+      <c r="Q27" s="60"/>
+      <c r="R27" s="60"/>
+      <c r="S27" s="60"/>
       <c r="Z27" s="59" t="s">
         <v>427</v>
       </c>
@@ -3696,21 +3795,21 @@
       <c r="J28" s="33" t="s">
         <v>434</v>
       </c>
-      <c r="K28" s="88" t="s">
+      <c r="K28" s="60" t="s">
         <v>425</v>
       </c>
-      <c r="L28" s="88" t="s">
+      <c r="L28" s="60" t="s">
         <v>433</v>
       </c>
-      <c r="M28" s="88"/>
-      <c r="N28" s="88" t="s">
+      <c r="M28" s="60"/>
+      <c r="N28" s="60" t="s">
         <v>435</v>
       </c>
-      <c r="O28" s="88"/>
-      <c r="P28" s="88"/>
-      <c r="Q28" s="88"/>
-      <c r="R28" s="88"/>
-      <c r="S28" s="88"/>
+      <c r="O28" s="60"/>
+      <c r="P28" s="60"/>
+      <c r="Q28" s="60"/>
+      <c r="R28" s="60"/>
+      <c r="S28" s="60"/>
       <c r="Z28" s="59" t="s">
         <v>436</v>
       </c>
@@ -3740,21 +3839,21 @@
       <c r="J29" s="33" t="s">
         <v>442</v>
       </c>
-      <c r="K29" s="88" t="s">
+      <c r="K29" s="60" t="s">
         <v>425</v>
       </c>
-      <c r="L29" s="88" t="s">
+      <c r="L29" s="60" t="s">
         <v>441</v>
       </c>
-      <c r="M29" s="88"/>
-      <c r="N29" s="88" t="s">
+      <c r="M29" s="60"/>
+      <c r="N29" s="60" t="s">
         <v>250</v>
       </c>
-      <c r="O29" s="88"/>
-      <c r="P29" s="88"/>
-      <c r="Q29" s="88"/>
-      <c r="R29" s="88"/>
-      <c r="S29" s="88"/>
+      <c r="O29" s="60"/>
+      <c r="P29" s="60"/>
+      <c r="Q29" s="60"/>
+      <c r="R29" s="60"/>
+      <c r="S29" s="60"/>
       <c r="Z29" s="59" t="s">
         <v>443</v>
       </c>
@@ -3772,15 +3871,15 @@
       <c r="E30" s="33" t="s">
         <v>446</v>
       </c>
-      <c r="K30" s="88"/>
-      <c r="L30" s="88"/>
-      <c r="M30" s="88"/>
-      <c r="N30" s="88"/>
-      <c r="O30" s="88"/>
-      <c r="P30" s="88"/>
-      <c r="Q30" s="88"/>
-      <c r="R30" s="88"/>
-      <c r="S30" s="88"/>
+      <c r="K30" s="60"/>
+      <c r="L30" s="60"/>
+      <c r="M30" s="60"/>
+      <c r="N30" s="60"/>
+      <c r="O30" s="60"/>
+      <c r="P30" s="60"/>
+      <c r="Q30" s="60"/>
+      <c r="R30" s="60"/>
+      <c r="S30" s="60"/>
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A31" s="33">
@@ -3798,15 +3897,15 @@
       <c r="H31" s="33" t="s">
         <v>447</v>
       </c>
-      <c r="K31" s="88"/>
-      <c r="L31" s="88"/>
-      <c r="M31" s="88"/>
-      <c r="N31" s="88"/>
-      <c r="O31" s="88"/>
-      <c r="P31" s="88"/>
-      <c r="Q31" s="88"/>
-      <c r="R31" s="88"/>
-      <c r="S31" s="88"/>
+      <c r="K31" s="60"/>
+      <c r="L31" s="60"/>
+      <c r="M31" s="60"/>
+      <c r="N31" s="60"/>
+      <c r="O31" s="60"/>
+      <c r="P31" s="60"/>
+      <c r="Q31" s="60"/>
+      <c r="R31" s="60"/>
+      <c r="S31" s="60"/>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A32" s="33">
@@ -3825,7 +3924,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="33">
         <v>99218793</v>
       </c>
@@ -3840,6 +3939,349 @@
       </c>
       <c r="H33" s="33" t="s">
         <v>447</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="33">
+        <v>96000001</v>
+      </c>
+      <c r="B34" s="33" t="s">
+        <v>451</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>313</v>
+      </c>
+      <c r="G34" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H34" s="33" t="s">
+        <v>319</v>
+      </c>
+      <c r="N34" s="33" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="33">
+        <v>96000002</v>
+      </c>
+      <c r="B35" s="33" t="s">
+        <v>452</v>
+      </c>
+      <c r="E35" s="33" t="s">
+        <v>313</v>
+      </c>
+      <c r="G35" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H35" s="33" t="s">
+        <v>319</v>
+      </c>
+      <c r="N35" s="33" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="33">
+        <v>96000003</v>
+      </c>
+      <c r="B36" s="33" t="s">
+        <v>454</v>
+      </c>
+      <c r="E36" s="33" t="s">
+        <v>302</v>
+      </c>
+      <c r="G36" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H36" s="33" t="s">
+        <v>308</v>
+      </c>
+      <c r="N36" s="33" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="33">
+        <v>96000004</v>
+      </c>
+      <c r="B37" s="33" t="s">
+        <v>456</v>
+      </c>
+      <c r="E37" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G37" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H37" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="N37" s="33" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="33">
+        <v>96000005</v>
+      </c>
+      <c r="B38" s="33" t="s">
+        <v>459</v>
+      </c>
+      <c r="E38" s="33" t="s">
+        <v>302</v>
+      </c>
+      <c r="G38" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H38" s="33" t="s">
+        <v>308</v>
+      </c>
+      <c r="N38" s="33" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="33">
+        <v>96000006</v>
+      </c>
+      <c r="B39" s="33" t="s">
+        <v>461</v>
+      </c>
+      <c r="E39" s="33" t="s">
+        <v>317</v>
+      </c>
+      <c r="G39" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H39" s="33" t="s">
+        <v>462</v>
+      </c>
+      <c r="N39" s="33" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A40" s="33">
+        <v>96000007</v>
+      </c>
+      <c r="B40" s="33" t="s">
+        <v>463</v>
+      </c>
+      <c r="E40" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="G40" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H40" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="N40" s="33" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A41" s="33">
+        <v>96000008</v>
+      </c>
+      <c r="B41" s="33" t="s">
+        <v>464</v>
+      </c>
+      <c r="E41" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="G41" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H41" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="L41" s="33" t="s">
+        <v>465</v>
+      </c>
+      <c r="N41" s="33" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42" s="33">
+        <v>96000009</v>
+      </c>
+      <c r="B42" s="33" t="s">
+        <v>466</v>
+      </c>
+      <c r="E42" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H42" s="33" t="s">
+        <v>467</v>
+      </c>
+      <c r="N42" s="33" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43" s="33">
+        <v>96000010</v>
+      </c>
+      <c r="B43" s="33" t="s">
+        <v>469</v>
+      </c>
+      <c r="E43" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G43" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H43" s="33" t="s">
+        <v>470</v>
+      </c>
+      <c r="N43" s="33" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A44" s="33">
+        <v>96000011</v>
+      </c>
+      <c r="B44" s="33" t="s">
+        <v>471</v>
+      </c>
+      <c r="E44" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="G44" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H44" s="33" t="s">
+        <v>392</v>
+      </c>
+      <c r="N44" s="33" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45" s="33">
+        <v>96000012</v>
+      </c>
+      <c r="B45" s="33" t="s">
+        <v>473</v>
+      </c>
+      <c r="E45" s="33" t="s">
+        <v>317</v>
+      </c>
+      <c r="G45" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H45" s="33" t="s">
+        <v>297</v>
+      </c>
+      <c r="N45" s="33" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A46" s="33">
+        <v>96000013</v>
+      </c>
+      <c r="B46" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="E46" s="33" t="s">
+        <v>302</v>
+      </c>
+      <c r="G46" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H46" s="33" t="s">
+        <v>476</v>
+      </c>
+      <c r="N46" s="33" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47" s="33">
+        <v>96000014</v>
+      </c>
+      <c r="B47" s="33" t="s">
+        <v>477</v>
+      </c>
+      <c r="E47" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G47" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H47" s="33" t="s">
+        <v>478</v>
+      </c>
+      <c r="N47" s="33" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48" s="33">
+        <v>96000015</v>
+      </c>
+      <c r="B48" s="33" t="s">
+        <v>479</v>
+      </c>
+      <c r="E48" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H48" s="33" t="s">
+        <v>480</v>
+      </c>
+      <c r="N48" s="33" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49" s="33">
+        <v>96000016</v>
+      </c>
+      <c r="B49" s="33" t="s">
+        <v>481</v>
+      </c>
+      <c r="E49" s="33" t="s">
+        <v>313</v>
+      </c>
+      <c r="G49" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H49" s="33" t="s">
+        <v>482</v>
+      </c>
+      <c r="N49" s="33" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="33">
+        <v>96000017</v>
+      </c>
+      <c r="B50" s="33" t="s">
+        <v>483</v>
+      </c>
+      <c r="E50" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G50" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H50" s="33" t="s">
+        <v>397</v>
+      </c>
+      <c r="N50" s="33" t="s">
+        <v>472</v>
       </c>
     </row>
   </sheetData>
@@ -5448,91 +5890,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64"/>
-      <c r="B1" s="64"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="68" t="s">
+      <c r="A1" s="65"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="69" t="s">
         <v>216</v>
       </c>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="71" t="s">
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72" t="s">
         <v>217</v>
       </c>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="74" t="s">
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="74"/>
+      <c r="P1" s="75" t="s">
         <v>216</v>
       </c>
-      <c r="Q1" s="75"/>
+      <c r="Q1" s="76"/>
       <c r="R1" s="6"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="64"/>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="76" t="s">
+      <c r="A2" s="65"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="77" t="s">
         <v>218</v>
       </c>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="79" t="s">
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="80" t="s">
         <v>219</v>
       </c>
-      <c r="K2" s="80"/>
-      <c r="L2" s="80"/>
-      <c r="M2" s="80"/>
-      <c r="N2" s="80"/>
-      <c r="O2" s="81"/>
-      <c r="P2" s="82" t="s">
+      <c r="K2" s="81"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="81"/>
+      <c r="N2" s="81"/>
+      <c r="O2" s="82"/>
+      <c r="P2" s="83" t="s">
         <v>220</v>
       </c>
-      <c r="Q2" s="83"/>
+      <c r="Q2" s="84"/>
       <c r="R2" s="5"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="64"/>
-      <c r="B3" s="64"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="84" t="s">
+      <c r="A3" s="65"/>
+      <c r="B3" s="65"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="85" t="s">
         <v>221</v>
       </c>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="86" t="s">
+      <c r="E3" s="86"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="86"/>
+      <c r="H3" s="87" t="s">
         <v>222</v>
       </c>
-      <c r="I3" s="87"/>
-      <c r="J3" s="84" t="s">
+      <c r="I3" s="88"/>
+      <c r="J3" s="85" t="s">
         <v>223</v>
       </c>
-      <c r="K3" s="85"/>
-      <c r="L3" s="85"/>
-      <c r="M3" s="85"/>
-      <c r="N3" s="85"/>
-      <c r="O3" s="87"/>
-      <c r="P3" s="60" t="s">
+      <c r="K3" s="86"/>
+      <c r="L3" s="86"/>
+      <c r="M3" s="86"/>
+      <c r="N3" s="86"/>
+      <c r="O3" s="88"/>
+      <c r="P3" s="61" t="s">
         <v>224</v>
       </c>
-      <c r="Q3" s="62" t="s">
+      <c r="Q3" s="63" t="s">
         <v>225</v>
       </c>
       <c r="R3" s="5"/>
     </row>
     <row r="4" spans="1:18" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="66"/>
-      <c r="B4" s="66"/>
-      <c r="C4" s="67"/>
+      <c r="A4" s="67"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="68"/>
       <c r="D4" s="9" t="s">
         <v>226</v>
       </c>
@@ -5569,8 +6011,8 @@
       <c r="O4" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="P4" s="61"/>
-      <c r="Q4" s="63"/>
+      <c r="P4" s="62"/>
+      <c r="Q4" s="64"/>
       <c r="R4" s="5"/>
     </row>
     <row r="5" spans="1:18" ht="240.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>